<commit_message>
refactor: update excel lookups, freeze header rows, and implement fallback markers
- **docs**: update `to_do.txt` to mark completed tasks across GUI and Excel processors[cite: 2].
- **excel**: add row-freezing via `init_freeze_row` in `excel_helper.py` and implement it in `money_excel.py` and `water_excel.py`[cite: 2].
- **excel**: enhance `find_last_value_row` in `excel_helper.py` to accept a boundary index (`last_find_row`) and adjust lookup calls[cite: 2].
- **json/converter**: implement default account marking fallback (`money_curreny_have_account_mark`) in `json_converter.py` if no modern "Money current have" entry is discovered[cite: 2].
- **style**: re-indent multiple project files to use a consistent 2-space indentation style instead of mixed 4-space tabs/indents[cite: 2].
</commit_message>
<xml_diff>
--- a/output/2026/money/backup.xlsx
+++ b/output/2026/money/backup.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1740" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2017" uniqueCount="203">
   <si>
     <t>Date</t>
   </si>
@@ -583,6 +583,54 @@
   <si>
     <t>114</t>
   </si>
+  <si>
+    <t>13/07/2026</t>
+  </si>
+  <si>
+    <t>Piggy-play</t>
+  </si>
+  <si>
+    <t>70.5</t>
+  </si>
+  <si>
+    <t>14/07/2026</t>
+  </si>
+  <si>
+    <t>45.5</t>
+  </si>
+  <si>
+    <t>65</t>
+  </si>
+  <si>
+    <t>123</t>
+  </si>
+  <si>
+    <t>15/07/2026</t>
+  </si>
+  <si>
+    <t>13.44</t>
+  </si>
+  <si>
+    <t>work</t>
+  </si>
+  <si>
+    <t>16/07/2026</t>
+  </si>
+  <si>
+    <t>83</t>
+  </si>
+  <si>
+    <t>17/07/2026</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>27.13</t>
+  </si>
+  <si>
+    <t>95</t>
+  </si>
 </sst>
 </file>
 
@@ -632,7 +680,7 @@
       <name val="Book Antiqua"/>
     </font>
   </fonts>
-  <fills count="133">
+  <fills count="163">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1305,8 +1353,158 @@
         <fgColor rgb="FF92D050"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEBF1DE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6E0B4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2DCDB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCE6F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC5D9F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFDE9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE4DFEC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDD9C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFBDBD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEBF1DE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6E0B4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2DCDB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCE6F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC5D9F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFDE9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE4DFEC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDD9C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFBDBD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEBF1DE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6E0B4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2DCDB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCE6F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC5D9F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFDE9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE4DFEC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDD9C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFBDBD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="317">
+  <borders count="389">
     <border>
       <left/>
       <right/>
@@ -4238,6 +4436,1086 @@
     <border>
       <left/>
       <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
       <top style="medium">
         <color auto="1"/>
       </top>
@@ -6051,7 +7329,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2007">
+  <cellXfs count="2441">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -8219,60 +9497,494 @@
     <xf numFmtId="0" fontId="0" fillId="131" borderId="316" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="131" borderId="315" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="132" borderId="313" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="7" borderId="289" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="317" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="133" borderId="318" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="133" borderId="319" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="134" borderId="318" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="134" borderId="319" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="135" borderId="318" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="135" borderId="319" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="136" borderId="318" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="136" borderId="319" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="137" borderId="318" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="137" borderId="319" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="138" borderId="318" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="138" borderId="319" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="139" borderId="318" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="139" borderId="319" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="140" borderId="318" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="140" borderId="319" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="141" borderId="318" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="141" borderId="320" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="141" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="142" borderId="317" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="321" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="133" borderId="322" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="133" borderId="323" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="134" borderId="322" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="134" borderId="323" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="135" borderId="322" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="135" borderId="323" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="136" borderId="322" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="136" borderId="323" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="137" borderId="322" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="137" borderId="323" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="138" borderId="322" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="138" borderId="323" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="139" borderId="322" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="139" borderId="323" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="140" borderId="322" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="140" borderId="323" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="141" borderId="322" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="141" borderId="324" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="141" borderId="323" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="142" borderId="321" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="136" borderId="322" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="136" borderId="323" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="137" borderId="322" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="137" borderId="323" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="135" borderId="322" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="135" borderId="323" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="140" borderId="322" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="140" borderId="323" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="141" borderId="322" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="141" borderId="324" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="325" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="133" borderId="326" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="133" borderId="327" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="134" borderId="326" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="134" borderId="327" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="135" borderId="326" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="135" borderId="327" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="136" borderId="326" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="136" borderId="327" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="137" borderId="326" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="137" borderId="327" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="138" borderId="326" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="138" borderId="327" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="139" borderId="326" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="139" borderId="327" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="140" borderId="326" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="140" borderId="327" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="141" borderId="326" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="141" borderId="328" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="141" borderId="327" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="142" borderId="325" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="329" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="133" borderId="330" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="133" borderId="331" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="134" borderId="330" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="134" borderId="331" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="135" borderId="330" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="135" borderId="331" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="136" borderId="330" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="136" borderId="331" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="137" borderId="330" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="137" borderId="331" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="138" borderId="330" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="138" borderId="331" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="139" borderId="330" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="139" borderId="331" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="140" borderId="330" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="140" borderId="331" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="141" borderId="330" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="141" borderId="332" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="141" borderId="331" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="142" borderId="329" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="333" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="133" borderId="334" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="133" borderId="335" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="134" borderId="334" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="134" borderId="335" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="135" borderId="334" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="135" borderId="335" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="136" borderId="334" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="136" borderId="335" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="137" borderId="334" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="137" borderId="335" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="138" borderId="334" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="138" borderId="335" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="139" borderId="334" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="139" borderId="335" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="140" borderId="334" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="140" borderId="335" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="141" borderId="334" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="141" borderId="336" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="141" borderId="335" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="142" borderId="333" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="337" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="133" borderId="338" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="133" borderId="339" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="134" borderId="338" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="134" borderId="339" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="135" borderId="338" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="135" borderId="339" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="136" borderId="338" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="136" borderId="339" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="137" borderId="338" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="137" borderId="339" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="138" borderId="338" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="138" borderId="339" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="139" borderId="338" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="139" borderId="339" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="140" borderId="338" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="140" borderId="339" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="141" borderId="338" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="141" borderId="340" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="141" borderId="339" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="142" borderId="337" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="341" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="143" borderId="342" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="143" borderId="343" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="144" borderId="342" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="144" borderId="343" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="145" borderId="342" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="145" borderId="343" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="146" borderId="342" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="146" borderId="343" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="147" borderId="342" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="147" borderId="343" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="148" borderId="342" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="148" borderId="343" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="149" borderId="342" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="149" borderId="343" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="150" borderId="342" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="150" borderId="343" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="151" borderId="342" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="151" borderId="344" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="151" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="152" borderId="341" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="345" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="143" borderId="346" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="143" borderId="347" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="144" borderId="346" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="144" borderId="347" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="145" borderId="346" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="145" borderId="347" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="146" borderId="346" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="146" borderId="347" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="147" borderId="346" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="147" borderId="347" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="148" borderId="346" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="148" borderId="347" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="149" borderId="346" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="149" borderId="347" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="150" borderId="346" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="150" borderId="347" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="151" borderId="346" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="151" borderId="348" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="151" borderId="347" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="152" borderId="345" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="146" borderId="346" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="146" borderId="347" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="147" borderId="346" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="147" borderId="347" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="145" borderId="346" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="145" borderId="347" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="150" borderId="346" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="150" borderId="347" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="151" borderId="346" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="151" borderId="348" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="349" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="143" borderId="350" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="143" borderId="351" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="144" borderId="350" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="144" borderId="351" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="145" borderId="350" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="145" borderId="351" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="146" borderId="350" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="146" borderId="351" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="147" borderId="350" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="147" borderId="351" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="148" borderId="350" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="148" borderId="351" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="149" borderId="350" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="149" borderId="351" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="150" borderId="350" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="150" borderId="351" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="151" borderId="350" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="151" borderId="352" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="151" borderId="351" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="152" borderId="349" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="353" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="143" borderId="354" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="143" borderId="355" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="144" borderId="354" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="144" borderId="355" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="145" borderId="354" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="145" borderId="355" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="146" borderId="354" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="146" borderId="355" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="147" borderId="354" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="147" borderId="355" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="148" borderId="354" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="148" borderId="355" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="149" borderId="354" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="149" borderId="355" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="150" borderId="354" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="150" borderId="355" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="151" borderId="354" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="151" borderId="356" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="151" borderId="355" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="152" borderId="353" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="357" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="143" borderId="358" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="143" borderId="359" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="144" borderId="358" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="144" borderId="359" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="145" borderId="358" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="145" borderId="359" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="146" borderId="358" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="146" borderId="359" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="147" borderId="358" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="147" borderId="359" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="148" borderId="358" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="148" borderId="359" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="149" borderId="358" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="149" borderId="359" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="150" borderId="358" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="150" borderId="359" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="151" borderId="358" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="151" borderId="360" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="151" borderId="359" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="152" borderId="357" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="145" borderId="342" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="145" borderId="343" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="146" borderId="342" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="146" borderId="343" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="147" borderId="342" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="147" borderId="343" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="150" borderId="342" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="150" borderId="343" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="151" borderId="342" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="151" borderId="344" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="361" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="143" borderId="362" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="143" borderId="363" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="144" borderId="362" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="144" borderId="363" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="145" borderId="362" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="145" borderId="363" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="146" borderId="362" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="146" borderId="363" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="147" borderId="362" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="147" borderId="363" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="148" borderId="362" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="148" borderId="363" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="149" borderId="362" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="149" borderId="363" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="150" borderId="362" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="150" borderId="363" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="151" borderId="362" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="151" borderId="364" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="151" borderId="363" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="152" borderId="361" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="365" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="153" borderId="366" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="153" borderId="367" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="154" borderId="366" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="154" borderId="367" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="155" borderId="366" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="155" borderId="367" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="156" borderId="366" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="156" borderId="367" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="157" borderId="366" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="157" borderId="367" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="158" borderId="366" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="158" borderId="367" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="159" borderId="366" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="159" borderId="367" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="160" borderId="366" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="160" borderId="367" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="161" borderId="366" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="161" borderId="368" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="161" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="162" borderId="365" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="369" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="153" borderId="370" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="153" borderId="371" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="154" borderId="370" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="154" borderId="371" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="155" borderId="370" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="155" borderId="371" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="156" borderId="370" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="156" borderId="371" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="157" borderId="370" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="157" borderId="371" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="158" borderId="370" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="158" borderId="371" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="159" borderId="370" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="159" borderId="371" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="160" borderId="370" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="160" borderId="371" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="161" borderId="370" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="161" borderId="372" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="161" borderId="371" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="162" borderId="369" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="155" borderId="370" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="155" borderId="371" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="160" borderId="370" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="160" borderId="371" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="161" borderId="370" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="161" borderId="372" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="156" borderId="370" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="156" borderId="371" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="157" borderId="370" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="157" borderId="371" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="373" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="153" borderId="374" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="153" borderId="375" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="154" borderId="374" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="154" borderId="375" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="155" borderId="374" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="155" borderId="375" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="156" borderId="374" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="156" borderId="375" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="157" borderId="374" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="157" borderId="375" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="158" borderId="374" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="158" borderId="375" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="159" borderId="374" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="159" borderId="375" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="160" borderId="374" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="160" borderId="375" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="161" borderId="374" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="161" borderId="376" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="161" borderId="375" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="162" borderId="373" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="377" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="153" borderId="378" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="153" borderId="379" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="154" borderId="378" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="154" borderId="379" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="155" borderId="378" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="155" borderId="379" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="156" borderId="378" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="156" borderId="379" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="157" borderId="378" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="157" borderId="379" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="158" borderId="378" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="158" borderId="379" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="159" borderId="378" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="159" borderId="379" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="160" borderId="378" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="160" borderId="379" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="161" borderId="378" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="161" borderId="380" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="161" borderId="379" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="162" borderId="377" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="381" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="153" borderId="382" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="153" borderId="383" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="154" borderId="382" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="154" borderId="383" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="155" borderId="382" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="155" borderId="383" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="156" borderId="382" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="156" borderId="383" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="157" borderId="382" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="157" borderId="383" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="158" borderId="382" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="158" borderId="383" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="159" borderId="382" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="159" borderId="383" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="160" borderId="382" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="160" borderId="383" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="161" borderId="382" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="161" borderId="384" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="161" borderId="383" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="162" borderId="381" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="385" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="153" borderId="386" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="153" borderId="387" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="154" borderId="386" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="154" borderId="387" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="155" borderId="386" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="155" borderId="387" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="156" borderId="386" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="156" borderId="387" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="157" borderId="386" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="157" borderId="387" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="158" borderId="386" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="158" borderId="387" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="159" borderId="386" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="159" borderId="387" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="160" borderId="386" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="160" borderId="387" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="161" borderId="386" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="161" borderId="388" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="161" borderId="387" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="162" borderId="385" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="155" borderId="366" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="155" borderId="367" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="156" borderId="366" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="156" borderId="367" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="157" borderId="366" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="157" borderId="367" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="160" borderId="366" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="160" borderId="367" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="161" borderId="366" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="161" borderId="368" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="159" borderId="370" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="159" borderId="371" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="157" borderId="374" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="157" borderId="375" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="158" borderId="374" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="158" borderId="375" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="7" borderId="361" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="195" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="6" borderId="289" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="6" borderId="361" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="8" borderId="289" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="8" borderId="361" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="289" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="361" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="3" borderId="289" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="361" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="22" borderId="289" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="22" borderId="361" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="5" borderId="289" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="5" borderId="361" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="4" borderId="289" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="4" borderId="361" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="9" borderId="289" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="9" borderId="361" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="196" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="79" borderId="289" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="79" borderId="361" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="78" borderId="289" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="78" borderId="361" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="80" borderId="289" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="80" borderId="361" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="73" borderId="289" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="73" borderId="361" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="75" borderId="289" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="75" borderId="361" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="74" borderId="289" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="74" borderId="361" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="77" borderId="289" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="77" borderId="361" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="76" borderId="289" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="76" borderId="361" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="81" borderId="289" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="81" borderId="361" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -8596,8 +10308,8 @@
   <cols>
     <col min="1" max="1" width="9" style="2" customWidth="1"/>
     <col min="2" max="2" width="13.125" style="2" customWidth="1"/>
-    <col min="3" max="17" width="9" style="2" customWidth="1"/>
-    <col min="18" max="16384" width="9" style="2"/>
+    <col min="3" max="21" width="9" style="2" customWidth="1"/>
+    <col min="22" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:22" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
@@ -8605,43 +10317,43 @@
       <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1991" t="s">
+      <c r="C2" s="2425" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="1988"/>
-      <c r="E2" s="1993" t="s">
+      <c r="D2" s="2422"/>
+      <c r="E2" s="2427" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="1988"/>
-      <c r="G2" s="1992" t="s">
+      <c r="F2" s="2422"/>
+      <c r="G2" s="2426" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="1988"/>
-      <c r="I2" s="1995" t="s">
+      <c r="H2" s="2422"/>
+      <c r="I2" s="2429" t="s">
         <v>4</v>
       </c>
-      <c r="J2" s="1988"/>
-      <c r="K2" s="1994" t="s">
+      <c r="J2" s="2422"/>
+      <c r="K2" s="2428" t="s">
         <v>5</v>
       </c>
-      <c r="L2" s="1988"/>
-      <c r="M2" s="1989" t="s">
+      <c r="L2" s="2422"/>
+      <c r="M2" s="2423" t="s">
         <v>6</v>
       </c>
-      <c r="N2" s="1988"/>
-      <c r="O2" s="1987" t="s">
+      <c r="N2" s="2422"/>
+      <c r="O2" s="2421" t="s">
         <v>7</v>
       </c>
-      <c r="P2" s="1988"/>
-      <c r="Q2" s="1990" t="s">
+      <c r="P2" s="2422"/>
+      <c r="Q2" s="2424" t="s">
         <v>8</v>
       </c>
-      <c r="R2" s="1988"/>
-      <c r="S2" s="1996" t="s">
+      <c r="R2" s="2422"/>
+      <c r="S2" s="2430" t="s">
         <v>9</v>
       </c>
-      <c r="T2" s="1997"/>
-      <c r="U2" s="1988"/>
+      <c r="T2" s="2431"/>
+      <c r="U2" s="2422"/>
       <c r="V2" s="4" t="s">
         <v>10</v>
       </c>
@@ -16878,57 +18590,57 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:W126"/>
+  <dimension ref="B2:W180"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" style="1098" customWidth="1"/>
     <col min="2" max="2" width="14.5" style="1098" customWidth="1"/>
     <col min="3" max="22" width="12" style="1098" customWidth="1"/>
-    <col min="23" max="26" width="9" style="1098" customWidth="1"/>
-    <col min="27" max="16384" width="9" style="1098"/>
+    <col min="23" max="30" width="9" style="1098" customWidth="1"/>
+    <col min="31" max="16384" width="9" style="1098"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="1096" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="2001" t="s">
+      <c r="C2" s="2435" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="1988"/>
-      <c r="E2" s="2003" t="s">
+      <c r="D2" s="2422"/>
+      <c r="E2" s="2437" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="1988"/>
-      <c r="G2" s="2002" t="s">
+      <c r="F2" s="2422"/>
+      <c r="G2" s="2436" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="1988"/>
-      <c r="I2" s="2005" t="s">
+      <c r="H2" s="2422"/>
+      <c r="I2" s="2439" t="s">
         <v>4</v>
       </c>
-      <c r="J2" s="1988"/>
-      <c r="K2" s="2004" t="s">
+      <c r="J2" s="2422"/>
+      <c r="K2" s="2438" t="s">
         <v>132</v>
       </c>
-      <c r="L2" s="1988"/>
-      <c r="M2" s="1999" t="s">
+      <c r="L2" s="2422"/>
+      <c r="M2" s="2433" t="s">
         <v>6</v>
       </c>
-      <c r="N2" s="1988"/>
-      <c r="O2" s="1998" t="s">
+      <c r="N2" s="2422"/>
+      <c r="O2" s="2432" t="s">
         <v>7</v>
       </c>
-      <c r="P2" s="1988"/>
-      <c r="Q2" s="2000" t="s">
+      <c r="P2" s="2422"/>
+      <c r="Q2" s="2434" t="s">
         <v>8</v>
       </c>
-      <c r="R2" s="1988"/>
-      <c r="S2" s="2006" t="s">
+      <c r="R2" s="2422"/>
+      <c r="S2" s="2440" t="s">
         <v>9</v>
       </c>
-      <c r="T2" s="1997"/>
-      <c r="U2" s="1988"/>
+      <c r="T2" s="2431"/>
+      <c r="U2" s="2422"/>
       <c r="V2" s="1097" t="s">
         <v>10</v>
       </c>
@@ -21006,7 +22718,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="113" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B113" s="1841" t="s">
         <v>183</v>
       </c>
@@ -21039,7 +22751,7 @@
       <c r="U113" s="1860"/>
       <c r="V113" s="1861"/>
     </row>
-    <row r="114" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B114" s="1862"/>
       <c r="C114" s="1863"/>
       <c r="D114" s="1864"/>
@@ -21070,7 +22782,7 @@
       <c r="U114" s="1881"/>
       <c r="V114" s="1882"/>
     </row>
-    <row r="115" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B115" s="1883"/>
       <c r="C115" s="1884"/>
       <c r="D115" s="1885"/>
@@ -21105,7 +22817,7 @@
       <c r="U115" s="1902"/>
       <c r="V115" s="1903"/>
     </row>
-    <row r="116" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B116" s="1904" t="s">
         <v>18</v>
       </c>
@@ -21156,7 +22868,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="117" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B117" s="1925" t="s">
         <v>20</v>
       </c>
@@ -21189,7 +22901,7 @@
       <c r="U117" s="1944"/>
       <c r="V117" s="1945"/>
     </row>
-    <row r="118" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B118" s="1841" t="s">
         <v>185</v>
       </c>
@@ -21226,7 +22938,7 @@
       <c r="U118" s="1860"/>
       <c r="V118" s="1861"/>
     </row>
-    <row r="119" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B119" s="1862"/>
       <c r="C119" s="1863"/>
       <c r="D119" s="1864"/>
@@ -21257,7 +22969,7 @@
       <c r="U119" s="1881"/>
       <c r="V119" s="1882"/>
     </row>
-    <row r="120" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B120" s="1862"/>
       <c r="C120" s="1863"/>
       <c r="D120" s="1864"/>
@@ -21292,7 +23004,7 @@
       <c r="U120" s="1881"/>
       <c r="V120" s="1882"/>
     </row>
-    <row r="121" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B121" s="1862"/>
       <c r="C121" s="1863"/>
       <c r="D121" s="1864"/>
@@ -21323,7 +23035,7 @@
       <c r="U121" s="1881"/>
       <c r="V121" s="1882"/>
     </row>
-    <row r="122" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B122" s="1862"/>
       <c r="C122" s="1863"/>
       <c r="D122" s="1864"/>
@@ -21357,8 +23069,11 @@
       </c>
       <c r="U122" s="1881"/>
       <c r="V122" s="1882"/>
-    </row>
-    <row r="123" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="W122" s="1098" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="123" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B123" s="1883"/>
       <c r="C123" s="1884"/>
       <c r="D123" s="1885"/>
@@ -21393,7 +23108,7 @@
       <c r="U123" s="1902"/>
       <c r="V123" s="1903"/>
     </row>
-    <row r="124" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B124" s="1904" t="s">
         <v>18</v>
       </c>
@@ -21444,7 +23159,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="125" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B125" s="1925" t="s">
         <v>20</v>
       </c>
@@ -21477,7 +23192,7 @@
       <c r="U125" s="1944"/>
       <c r="V125" s="1945"/>
     </row>
-    <row r="126" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="126" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B126" s="1966" t="s">
         <v>21</v>
       </c>
@@ -21531,6 +23246,2028 @@
         <v>12241.05</v>
       </c>
       <c r="V126" s="1986" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="127" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B127" s="1987" t="s">
+        <v>187</v>
+      </c>
+      <c r="C127" s="1988"/>
+      <c r="D127" s="1989"/>
+      <c r="E127" s="1990"/>
+      <c r="F127" s="1991"/>
+      <c r="G127" s="1992" t="s">
+        <v>5</v>
+      </c>
+      <c r="H127" s="1993" t="s">
+        <v>101</v>
+      </c>
+      <c r="I127" s="1994"/>
+      <c r="J127" s="1995"/>
+      <c r="K127" s="1996" t="s">
+        <v>101</v>
+      </c>
+      <c r="L127" s="1997" t="s">
+        <v>28</v>
+      </c>
+      <c r="M127" s="1998"/>
+      <c r="N127" s="1999"/>
+      <c r="O127" s="2000"/>
+      <c r="P127" s="2001"/>
+      <c r="Q127" s="2002"/>
+      <c r="R127" s="2003"/>
+      <c r="S127" s="2004"/>
+      <c r="T127" s="2005"/>
+      <c r="U127" s="2006"/>
+      <c r="V127" s="2007"/>
+    </row>
+    <row r="128" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B128" s="2008"/>
+      <c r="C128" s="2009"/>
+      <c r="D128" s="2010"/>
+      <c r="E128" s="2011"/>
+      <c r="F128" s="2012"/>
+      <c r="G128" s="2013"/>
+      <c r="H128" s="2014"/>
+      <c r="I128" s="2015"/>
+      <c r="J128" s="2016"/>
+      <c r="K128" s="2017" t="s">
+        <v>44</v>
+      </c>
+      <c r="L128" s="2018" t="s">
+        <v>101</v>
+      </c>
+      <c r="M128" s="2019"/>
+      <c r="N128" s="2020"/>
+      <c r="O128" s="2021"/>
+      <c r="P128" s="2022"/>
+      <c r="Q128" s="2023" t="s">
+        <v>44</v>
+      </c>
+      <c r="R128" s="2024" t="s">
+        <v>101</v>
+      </c>
+      <c r="S128" s="2025" t="s">
+        <v>44</v>
+      </c>
+      <c r="T128" s="2026" t="s">
+        <v>101</v>
+      </c>
+      <c r="U128" s="2027"/>
+      <c r="V128" s="2028"/>
+    </row>
+    <row r="129" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B129" s="2008"/>
+      <c r="C129" s="2009"/>
+      <c r="D129" s="2010"/>
+      <c r="E129" s="2011"/>
+      <c r="F129" s="2012"/>
+      <c r="G129" s="2013"/>
+      <c r="H129" s="2014"/>
+      <c r="I129" s="2029" t="s">
+        <v>188</v>
+      </c>
+      <c r="J129" s="2030" t="s">
+        <v>150</v>
+      </c>
+      <c r="K129" s="2031"/>
+      <c r="L129" s="2032"/>
+      <c r="M129" s="2019"/>
+      <c r="N129" s="2020"/>
+      <c r="O129" s="2021"/>
+      <c r="P129" s="2022"/>
+      <c r="Q129" s="2023" t="s">
+        <v>188</v>
+      </c>
+      <c r="R129" s="2024" t="s">
+        <v>150</v>
+      </c>
+      <c r="S129" s="2025" t="s">
+        <v>188</v>
+      </c>
+      <c r="T129" s="2026" t="s">
+        <v>150</v>
+      </c>
+      <c r="U129" s="2027"/>
+      <c r="V129" s="2028"/>
+      <c r="W129" s="1098" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="130" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B130" s="2008"/>
+      <c r="C130" s="2009"/>
+      <c r="D130" s="2010"/>
+      <c r="E130" s="2011"/>
+      <c r="F130" s="2012"/>
+      <c r="G130" s="2013"/>
+      <c r="H130" s="2014"/>
+      <c r="I130" s="2029" t="s">
+        <v>23</v>
+      </c>
+      <c r="J130" s="2030" t="s">
+        <v>48</v>
+      </c>
+      <c r="K130" s="2031"/>
+      <c r="L130" s="2032"/>
+      <c r="M130" s="2019"/>
+      <c r="N130" s="2020"/>
+      <c r="O130" s="2021"/>
+      <c r="P130" s="2022"/>
+      <c r="Q130" s="2023" t="s">
+        <v>23</v>
+      </c>
+      <c r="R130" s="2024" t="s">
+        <v>48</v>
+      </c>
+      <c r="S130" s="2025" t="s">
+        <v>23</v>
+      </c>
+      <c r="T130" s="2026" t="s">
+        <v>48</v>
+      </c>
+      <c r="U130" s="2027"/>
+      <c r="V130" s="2028"/>
+    </row>
+    <row r="131" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B131" s="2008"/>
+      <c r="C131" s="2009"/>
+      <c r="D131" s="2010"/>
+      <c r="E131" s="2011"/>
+      <c r="F131" s="2012"/>
+      <c r="G131" s="2033" t="s">
+        <v>5</v>
+      </c>
+      <c r="H131" s="2034" t="s">
+        <v>189</v>
+      </c>
+      <c r="I131" s="2015"/>
+      <c r="J131" s="2016"/>
+      <c r="K131" s="2017" t="s">
+        <v>189</v>
+      </c>
+      <c r="L131" s="2018" t="s">
+        <v>28</v>
+      </c>
+      <c r="M131" s="2019"/>
+      <c r="N131" s="2020"/>
+      <c r="O131" s="2021"/>
+      <c r="P131" s="2022"/>
+      <c r="Q131" s="2035"/>
+      <c r="R131" s="2036"/>
+      <c r="S131" s="2037"/>
+      <c r="T131" s="2038"/>
+      <c r="U131" s="2027"/>
+      <c r="V131" s="2028"/>
+    </row>
+    <row r="132" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B132" s="2008"/>
+      <c r="C132" s="2009"/>
+      <c r="D132" s="2010"/>
+      <c r="E132" s="2011"/>
+      <c r="F132" s="2012"/>
+      <c r="G132" s="2013"/>
+      <c r="H132" s="2014"/>
+      <c r="I132" s="2015"/>
+      <c r="J132" s="2016"/>
+      <c r="K132" s="2017" t="s">
+        <v>46</v>
+      </c>
+      <c r="L132" s="2018" t="s">
+        <v>189</v>
+      </c>
+      <c r="M132" s="2019"/>
+      <c r="N132" s="2020"/>
+      <c r="O132" s="2021"/>
+      <c r="P132" s="2022"/>
+      <c r="Q132" s="2023" t="s">
+        <v>46</v>
+      </c>
+      <c r="R132" s="2024" t="s">
+        <v>189</v>
+      </c>
+      <c r="S132" s="2025" t="s">
+        <v>46</v>
+      </c>
+      <c r="T132" s="2026" t="s">
+        <v>189</v>
+      </c>
+      <c r="U132" s="2027"/>
+      <c r="V132" s="2028"/>
+      <c r="W132" s="1098" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="133" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B133" s="2039"/>
+      <c r="C133" s="2040"/>
+      <c r="D133" s="2041"/>
+      <c r="E133" s="2042"/>
+      <c r="F133" s="2043"/>
+      <c r="G133" s="2044"/>
+      <c r="H133" s="2045"/>
+      <c r="I133" s="2046" t="s">
+        <v>23</v>
+      </c>
+      <c r="J133" s="2047" t="s">
+        <v>48</v>
+      </c>
+      <c r="K133" s="2048"/>
+      <c r="L133" s="2049"/>
+      <c r="M133" s="2050"/>
+      <c r="N133" s="2051"/>
+      <c r="O133" s="2052"/>
+      <c r="P133" s="2053"/>
+      <c r="Q133" s="2054" t="s">
+        <v>23</v>
+      </c>
+      <c r="R133" s="2055" t="s">
+        <v>48</v>
+      </c>
+      <c r="S133" s="2056" t="s">
+        <v>23</v>
+      </c>
+      <c r="T133" s="2057" t="s">
+        <v>48</v>
+      </c>
+      <c r="U133" s="2058"/>
+      <c r="V133" s="2059"/>
+    </row>
+    <row r="134" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B134" s="2060" t="s">
+        <v>18</v>
+      </c>
+      <c r="C134" s="2061">
+        <v>60</v>
+      </c>
+      <c r="D134" s="2062"/>
+      <c r="E134" s="2063">
+        <v>32.799999999999997</v>
+      </c>
+      <c r="F134" s="2064"/>
+      <c r="G134" s="2065">
+        <v>11713.17</v>
+      </c>
+      <c r="H134" s="2066"/>
+      <c r="I134" s="2067">
+        <v>280.89999999999998</v>
+      </c>
+      <c r="J134" s="2068"/>
+      <c r="K134" s="2069">
+        <v>0</v>
+      </c>
+      <c r="L134" s="2070"/>
+      <c r="M134" s="2071">
+        <v>48.48</v>
+      </c>
+      <c r="N134" s="2072"/>
+      <c r="O134" s="2073">
+        <v>0</v>
+      </c>
+      <c r="P134" s="2074"/>
+      <c r="Q134" s="2075">
+        <v>0</v>
+      </c>
+      <c r="R134" s="2076">
+        <v>105.7</v>
+      </c>
+      <c r="S134" s="2077">
+        <v>0</v>
+      </c>
+      <c r="T134" s="2078">
+        <v>105.7</v>
+      </c>
+      <c r="U134" s="2079">
+        <v>12135.35</v>
+      </c>
+      <c r="V134" s="2080" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="135" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B135" s="2081" t="s">
+        <v>20</v>
+      </c>
+      <c r="C135" s="2082"/>
+      <c r="D135" s="2083"/>
+      <c r="E135" s="2084"/>
+      <c r="F135" s="2085"/>
+      <c r="G135" s="2086"/>
+      <c r="H135" s="2087"/>
+      <c r="I135" s="2088"/>
+      <c r="J135" s="2089"/>
+      <c r="K135" s="2090"/>
+      <c r="L135" s="2091"/>
+      <c r="M135" s="2092"/>
+      <c r="N135" s="2093"/>
+      <c r="O135" s="2094"/>
+      <c r="P135" s="2095"/>
+      <c r="Q135" s="2096">
+        <v>0</v>
+      </c>
+      <c r="R135" s="2097">
+        <v>2185.48</v>
+      </c>
+      <c r="S135" s="2098">
+        <v>3700</v>
+      </c>
+      <c r="T135" s="2099">
+        <v>2685.48</v>
+      </c>
+      <c r="U135" s="2100"/>
+      <c r="V135" s="2101"/>
+    </row>
+    <row r="136" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B136" s="2102" t="s">
+        <v>21</v>
+      </c>
+      <c r="C136" s="2103">
+        <v>60</v>
+      </c>
+      <c r="D136" s="2104" t="s">
+        <v>19</v>
+      </c>
+      <c r="E136" s="2105">
+        <v>32.799999999999997</v>
+      </c>
+      <c r="F136" s="2106" t="s">
+        <v>19</v>
+      </c>
+      <c r="G136" s="2107">
+        <v>11713.17</v>
+      </c>
+      <c r="H136" s="2108" t="s">
+        <v>19</v>
+      </c>
+      <c r="I136" s="2109">
+        <v>280.89999999999998</v>
+      </c>
+      <c r="J136" s="2110" t="s">
+        <v>19</v>
+      </c>
+      <c r="K136" s="2111">
+        <v>0</v>
+      </c>
+      <c r="L136" s="2112" t="s">
+        <v>19</v>
+      </c>
+      <c r="M136" s="2113">
+        <v>48.48</v>
+      </c>
+      <c r="N136" s="2114" t="s">
+        <v>19</v>
+      </c>
+      <c r="O136" s="2115">
+        <v>0</v>
+      </c>
+      <c r="P136" s="2116" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q136" s="2117"/>
+      <c r="R136" s="2118"/>
+      <c r="S136" s="2119"/>
+      <c r="T136" s="2120"/>
+      <c r="U136" s="2121">
+        <v>12135.35</v>
+      </c>
+      <c r="V136" s="2122" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="137" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B137" s="2123" t="s">
+        <v>190</v>
+      </c>
+      <c r="C137" s="2124"/>
+      <c r="D137" s="2125"/>
+      <c r="E137" s="2126"/>
+      <c r="F137" s="2127"/>
+      <c r="G137" s="2128" t="s">
+        <v>5</v>
+      </c>
+      <c r="H137" s="2129" t="s">
+        <v>191</v>
+      </c>
+      <c r="I137" s="2130"/>
+      <c r="J137" s="2131"/>
+      <c r="K137" s="2132" t="s">
+        <v>191</v>
+      </c>
+      <c r="L137" s="2133" t="s">
+        <v>28</v>
+      </c>
+      <c r="M137" s="2134"/>
+      <c r="N137" s="2135"/>
+      <c r="O137" s="2136"/>
+      <c r="P137" s="2137"/>
+      <c r="Q137" s="2138"/>
+      <c r="R137" s="2139"/>
+      <c r="S137" s="2140"/>
+      <c r="T137" s="2141"/>
+      <c r="U137" s="2142"/>
+      <c r="V137" s="2143"/>
+    </row>
+    <row r="138" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B138" s="2144"/>
+      <c r="C138" s="2145"/>
+      <c r="D138" s="2146"/>
+      <c r="E138" s="2147"/>
+      <c r="F138" s="2148"/>
+      <c r="G138" s="2149"/>
+      <c r="H138" s="2150"/>
+      <c r="I138" s="2151"/>
+      <c r="J138" s="2152"/>
+      <c r="K138" s="2153" t="s">
+        <v>29</v>
+      </c>
+      <c r="L138" s="2154" t="s">
+        <v>191</v>
+      </c>
+      <c r="M138" s="2155"/>
+      <c r="N138" s="2156"/>
+      <c r="O138" s="2157"/>
+      <c r="P138" s="2158"/>
+      <c r="Q138" s="2159" t="s">
+        <v>29</v>
+      </c>
+      <c r="R138" s="2160" t="s">
+        <v>191</v>
+      </c>
+      <c r="S138" s="2161" t="s">
+        <v>29</v>
+      </c>
+      <c r="T138" s="2162" t="s">
+        <v>191</v>
+      </c>
+      <c r="U138" s="2163"/>
+      <c r="V138" s="2164"/>
+    </row>
+    <row r="139" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B139" s="2144"/>
+      <c r="C139" s="2145"/>
+      <c r="D139" s="2146"/>
+      <c r="E139" s="2147"/>
+      <c r="F139" s="2148"/>
+      <c r="G139" s="2149"/>
+      <c r="H139" s="2150"/>
+      <c r="I139" s="2165" t="s">
+        <v>50</v>
+      </c>
+      <c r="J139" s="2166" t="s">
+        <v>136</v>
+      </c>
+      <c r="K139" s="2167"/>
+      <c r="L139" s="2168"/>
+      <c r="M139" s="2155"/>
+      <c r="N139" s="2156"/>
+      <c r="O139" s="2157"/>
+      <c r="P139" s="2158"/>
+      <c r="Q139" s="2159" t="s">
+        <v>50</v>
+      </c>
+      <c r="R139" s="2160" t="s">
+        <v>136</v>
+      </c>
+      <c r="S139" s="2161" t="s">
+        <v>50</v>
+      </c>
+      <c r="T139" s="2162" t="s">
+        <v>136</v>
+      </c>
+      <c r="U139" s="2163"/>
+      <c r="V139" s="2164"/>
+    </row>
+    <row r="140" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B140" s="2144"/>
+      <c r="C140" s="2145"/>
+      <c r="D140" s="2146"/>
+      <c r="E140" s="2147"/>
+      <c r="F140" s="2148"/>
+      <c r="G140" s="2169" t="s">
+        <v>5</v>
+      </c>
+      <c r="H140" s="2170" t="s">
+        <v>192</v>
+      </c>
+      <c r="I140" s="2151"/>
+      <c r="J140" s="2152"/>
+      <c r="K140" s="2153" t="s">
+        <v>192</v>
+      </c>
+      <c r="L140" s="2154" t="s">
+        <v>28</v>
+      </c>
+      <c r="M140" s="2155"/>
+      <c r="N140" s="2156"/>
+      <c r="O140" s="2157"/>
+      <c r="P140" s="2158"/>
+      <c r="Q140" s="2171"/>
+      <c r="R140" s="2172"/>
+      <c r="S140" s="2173"/>
+      <c r="T140" s="2174"/>
+      <c r="U140" s="2163"/>
+      <c r="V140" s="2164"/>
+    </row>
+    <row r="141" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B141" s="2144"/>
+      <c r="C141" s="2145"/>
+      <c r="D141" s="2146"/>
+      <c r="E141" s="2147"/>
+      <c r="F141" s="2148"/>
+      <c r="G141" s="2149"/>
+      <c r="H141" s="2150"/>
+      <c r="I141" s="2151"/>
+      <c r="J141" s="2152"/>
+      <c r="K141" s="2153" t="s">
+        <v>46</v>
+      </c>
+      <c r="L141" s="2154" t="s">
+        <v>192</v>
+      </c>
+      <c r="M141" s="2155"/>
+      <c r="N141" s="2156"/>
+      <c r="O141" s="2157"/>
+      <c r="P141" s="2158"/>
+      <c r="Q141" s="2159" t="s">
+        <v>46</v>
+      </c>
+      <c r="R141" s="2160" t="s">
+        <v>192</v>
+      </c>
+      <c r="S141" s="2161" t="s">
+        <v>46</v>
+      </c>
+      <c r="T141" s="2162" t="s">
+        <v>192</v>
+      </c>
+      <c r="U141" s="2163"/>
+      <c r="V141" s="2164"/>
+    </row>
+    <row r="142" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B142" s="2144"/>
+      <c r="C142" s="2145"/>
+      <c r="D142" s="2146"/>
+      <c r="E142" s="2147"/>
+      <c r="F142" s="2148"/>
+      <c r="G142" s="2149"/>
+      <c r="H142" s="2150"/>
+      <c r="I142" s="2165" t="s">
+        <v>50</v>
+      </c>
+      <c r="J142" s="2166" t="s">
+        <v>165</v>
+      </c>
+      <c r="K142" s="2167"/>
+      <c r="L142" s="2168"/>
+      <c r="M142" s="2155"/>
+      <c r="N142" s="2156"/>
+      <c r="O142" s="2157"/>
+      <c r="P142" s="2158"/>
+      <c r="Q142" s="2159" t="s">
+        <v>50</v>
+      </c>
+      <c r="R142" s="2160" t="s">
+        <v>165</v>
+      </c>
+      <c r="S142" s="2161" t="s">
+        <v>50</v>
+      </c>
+      <c r="T142" s="2162" t="s">
+        <v>165</v>
+      </c>
+      <c r="U142" s="2163"/>
+      <c r="V142" s="2164"/>
+    </row>
+    <row r="143" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B143" s="2144"/>
+      <c r="C143" s="2145"/>
+      <c r="D143" s="2146"/>
+      <c r="E143" s="2147"/>
+      <c r="F143" s="2148"/>
+      <c r="G143" s="2149"/>
+      <c r="H143" s="2150"/>
+      <c r="I143" s="2165" t="s">
+        <v>94</v>
+      </c>
+      <c r="J143" s="2166" t="s">
+        <v>34</v>
+      </c>
+      <c r="K143" s="2167"/>
+      <c r="L143" s="2168"/>
+      <c r="M143" s="2155"/>
+      <c r="N143" s="2156"/>
+      <c r="O143" s="2157"/>
+      <c r="P143" s="2158"/>
+      <c r="Q143" s="2159" t="s">
+        <v>94</v>
+      </c>
+      <c r="R143" s="2160" t="s">
+        <v>34</v>
+      </c>
+      <c r="S143" s="2161" t="s">
+        <v>94</v>
+      </c>
+      <c r="T143" s="2162" t="s">
+        <v>34</v>
+      </c>
+      <c r="U143" s="2163"/>
+      <c r="V143" s="2164"/>
+    </row>
+    <row r="144" spans="2:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B144" s="2144"/>
+      <c r="C144" s="2145"/>
+      <c r="D144" s="2146"/>
+      <c r="E144" s="2147"/>
+      <c r="F144" s="2148"/>
+      <c r="G144" s="2169" t="s">
+        <v>33</v>
+      </c>
+      <c r="H144" s="2170" t="s">
+        <v>193</v>
+      </c>
+      <c r="I144" s="2151"/>
+      <c r="J144" s="2152"/>
+      <c r="K144" s="2167"/>
+      <c r="L144" s="2168"/>
+      <c r="M144" s="2155"/>
+      <c r="N144" s="2156"/>
+      <c r="O144" s="2157"/>
+      <c r="P144" s="2158"/>
+      <c r="Q144" s="2159" t="s">
+        <v>33</v>
+      </c>
+      <c r="R144" s="2160" t="s">
+        <v>193</v>
+      </c>
+      <c r="S144" s="2161" t="s">
+        <v>33</v>
+      </c>
+      <c r="T144" s="2162" t="s">
+        <v>193</v>
+      </c>
+      <c r="U144" s="2163"/>
+      <c r="V144" s="2164"/>
+      <c r="W144" s="1098" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="145" spans="2:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B145" s="2175"/>
+      <c r="C145" s="2176"/>
+      <c r="D145" s="2177"/>
+      <c r="E145" s="2178"/>
+      <c r="F145" s="2179"/>
+      <c r="G145" s="2180"/>
+      <c r="H145" s="2181"/>
+      <c r="I145" s="2182" t="s">
+        <v>23</v>
+      </c>
+      <c r="J145" s="2183" t="s">
+        <v>48</v>
+      </c>
+      <c r="K145" s="2184"/>
+      <c r="L145" s="2185"/>
+      <c r="M145" s="2186"/>
+      <c r="N145" s="2187"/>
+      <c r="O145" s="2188"/>
+      <c r="P145" s="2189"/>
+      <c r="Q145" s="2190" t="s">
+        <v>23</v>
+      </c>
+      <c r="R145" s="2191" t="s">
+        <v>48</v>
+      </c>
+      <c r="S145" s="2192" t="s">
+        <v>23</v>
+      </c>
+      <c r="T145" s="2193" t="s">
+        <v>48</v>
+      </c>
+      <c r="U145" s="2194"/>
+      <c r="V145" s="2195"/>
+    </row>
+    <row r="146" spans="2:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B146" s="2196" t="s">
+        <v>18</v>
+      </c>
+      <c r="C146" s="2197">
+        <v>60</v>
+      </c>
+      <c r="D146" s="2198"/>
+      <c r="E146" s="2199">
+        <v>32.799999999999997</v>
+      </c>
+      <c r="F146" s="2200"/>
+      <c r="G146" s="2201">
+        <v>11479.67</v>
+      </c>
+      <c r="H146" s="2202"/>
+      <c r="I146" s="2203">
+        <v>240</v>
+      </c>
+      <c r="J146" s="2204"/>
+      <c r="K146" s="2205">
+        <v>0</v>
+      </c>
+      <c r="L146" s="2206"/>
+      <c r="M146" s="2207">
+        <v>48.48</v>
+      </c>
+      <c r="N146" s="2208"/>
+      <c r="O146" s="2209">
+        <v>0</v>
+      </c>
+      <c r="P146" s="2210"/>
+      <c r="Q146" s="2211">
+        <v>0</v>
+      </c>
+      <c r="R146" s="2212">
+        <v>274.39999999999998</v>
+      </c>
+      <c r="S146" s="2213">
+        <v>0</v>
+      </c>
+      <c r="T146" s="2214">
+        <v>274.39999999999998</v>
+      </c>
+      <c r="U146" s="2215">
+        <v>11860.95</v>
+      </c>
+      <c r="V146" s="2216" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="147" spans="2:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B147" s="2217" t="s">
+        <v>20</v>
+      </c>
+      <c r="C147" s="2218"/>
+      <c r="D147" s="2219"/>
+      <c r="E147" s="2220"/>
+      <c r="F147" s="2221"/>
+      <c r="G147" s="2222"/>
+      <c r="H147" s="2223"/>
+      <c r="I147" s="2224"/>
+      <c r="J147" s="2225"/>
+      <c r="K147" s="2226"/>
+      <c r="L147" s="2227"/>
+      <c r="M147" s="2228"/>
+      <c r="N147" s="2229"/>
+      <c r="O147" s="2230"/>
+      <c r="P147" s="2231"/>
+      <c r="Q147" s="2232">
+        <v>0</v>
+      </c>
+      <c r="R147" s="2233">
+        <v>2459.88</v>
+      </c>
+      <c r="S147" s="2234">
+        <v>3700</v>
+      </c>
+      <c r="T147" s="2235">
+        <v>2959.88</v>
+      </c>
+      <c r="U147" s="2236"/>
+      <c r="V147" s="2237"/>
+    </row>
+    <row r="148" spans="2:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B148" s="2123" t="s">
+        <v>194</v>
+      </c>
+      <c r="C148" s="2124"/>
+      <c r="D148" s="2125"/>
+      <c r="E148" s="2126"/>
+      <c r="F148" s="2127"/>
+      <c r="G148" s="2238"/>
+      <c r="H148" s="2239"/>
+      <c r="I148" s="2240" t="s">
+        <v>23</v>
+      </c>
+      <c r="J148" s="2241" t="s">
+        <v>24</v>
+      </c>
+      <c r="K148" s="2242"/>
+      <c r="L148" s="2243"/>
+      <c r="M148" s="2134"/>
+      <c r="N148" s="2135"/>
+      <c r="O148" s="2136"/>
+      <c r="P148" s="2137"/>
+      <c r="Q148" s="2244" t="s">
+        <v>23</v>
+      </c>
+      <c r="R148" s="2245" t="s">
+        <v>24</v>
+      </c>
+      <c r="S148" s="2246" t="s">
+        <v>23</v>
+      </c>
+      <c r="T148" s="2247" t="s">
+        <v>24</v>
+      </c>
+      <c r="U148" s="2142"/>
+      <c r="V148" s="2143"/>
+    </row>
+    <row r="149" spans="2:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B149" s="2144"/>
+      <c r="C149" s="2145"/>
+      <c r="D149" s="2146"/>
+      <c r="E149" s="2147"/>
+      <c r="F149" s="2148"/>
+      <c r="G149" s="2169" t="s">
+        <v>5</v>
+      </c>
+      <c r="H149" s="2170" t="s">
+        <v>92</v>
+      </c>
+      <c r="I149" s="2151"/>
+      <c r="J149" s="2152"/>
+      <c r="K149" s="2153" t="s">
+        <v>92</v>
+      </c>
+      <c r="L149" s="2154" t="s">
+        <v>28</v>
+      </c>
+      <c r="M149" s="2155"/>
+      <c r="N149" s="2156"/>
+      <c r="O149" s="2157"/>
+      <c r="P149" s="2158"/>
+      <c r="Q149" s="2171"/>
+      <c r="R149" s="2172"/>
+      <c r="S149" s="2173"/>
+      <c r="T149" s="2174"/>
+      <c r="U149" s="2163"/>
+      <c r="V149" s="2164"/>
+    </row>
+    <row r="150" spans="2:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B150" s="2144"/>
+      <c r="C150" s="2145"/>
+      <c r="D150" s="2146"/>
+      <c r="E150" s="2147"/>
+      <c r="F150" s="2148"/>
+      <c r="G150" s="2149"/>
+      <c r="H150" s="2150"/>
+      <c r="I150" s="2151"/>
+      <c r="J150" s="2152"/>
+      <c r="K150" s="2153" t="s">
+        <v>93</v>
+      </c>
+      <c r="L150" s="2154" t="s">
+        <v>92</v>
+      </c>
+      <c r="M150" s="2155"/>
+      <c r="N150" s="2156"/>
+      <c r="O150" s="2157"/>
+      <c r="P150" s="2158"/>
+      <c r="Q150" s="2159" t="s">
+        <v>93</v>
+      </c>
+      <c r="R150" s="2160" t="s">
+        <v>92</v>
+      </c>
+      <c r="S150" s="2161" t="s">
+        <v>93</v>
+      </c>
+      <c r="T150" s="2162" t="s">
+        <v>92</v>
+      </c>
+      <c r="U150" s="2163"/>
+      <c r="V150" s="2164"/>
+    </row>
+    <row r="151" spans="2:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B151" s="2144"/>
+      <c r="C151" s="2145"/>
+      <c r="D151" s="2146"/>
+      <c r="E151" s="2147"/>
+      <c r="F151" s="2148"/>
+      <c r="G151" s="2149"/>
+      <c r="H151" s="2150"/>
+      <c r="I151" s="2165" t="s">
+        <v>25</v>
+      </c>
+      <c r="J151" s="2166" t="s">
+        <v>26</v>
+      </c>
+      <c r="K151" s="2167"/>
+      <c r="L151" s="2168"/>
+      <c r="M151" s="2155"/>
+      <c r="N151" s="2156"/>
+      <c r="O151" s="2157"/>
+      <c r="P151" s="2158"/>
+      <c r="Q151" s="2159" t="s">
+        <v>25</v>
+      </c>
+      <c r="R151" s="2160" t="s">
+        <v>26</v>
+      </c>
+      <c r="S151" s="2161" t="s">
+        <v>25</v>
+      </c>
+      <c r="T151" s="2162" t="s">
+        <v>26</v>
+      </c>
+      <c r="U151" s="2163"/>
+      <c r="V151" s="2164"/>
+    </row>
+    <row r="152" spans="2:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B152" s="2144"/>
+      <c r="C152" s="2145"/>
+      <c r="D152" s="2146"/>
+      <c r="E152" s="2147"/>
+      <c r="F152" s="2148"/>
+      <c r="G152" s="2169" t="s">
+        <v>5</v>
+      </c>
+      <c r="H152" s="2170" t="s">
+        <v>89</v>
+      </c>
+      <c r="I152" s="2151"/>
+      <c r="J152" s="2152"/>
+      <c r="K152" s="2153" t="s">
+        <v>89</v>
+      </c>
+      <c r="L152" s="2154" t="s">
+        <v>28</v>
+      </c>
+      <c r="M152" s="2155"/>
+      <c r="N152" s="2156"/>
+      <c r="O152" s="2157"/>
+      <c r="P152" s="2158"/>
+      <c r="Q152" s="2171"/>
+      <c r="R152" s="2172"/>
+      <c r="S152" s="2173"/>
+      <c r="T152" s="2174"/>
+      <c r="U152" s="2163"/>
+      <c r="V152" s="2164"/>
+    </row>
+    <row r="153" spans="2:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B153" s="2144"/>
+      <c r="C153" s="2145"/>
+      <c r="D153" s="2146"/>
+      <c r="E153" s="2147"/>
+      <c r="F153" s="2148"/>
+      <c r="G153" s="2149"/>
+      <c r="H153" s="2150"/>
+      <c r="I153" s="2151"/>
+      <c r="J153" s="2152"/>
+      <c r="K153" s="2153" t="s">
+        <v>46</v>
+      </c>
+      <c r="L153" s="2154" t="s">
+        <v>89</v>
+      </c>
+      <c r="M153" s="2155"/>
+      <c r="N153" s="2156"/>
+      <c r="O153" s="2157"/>
+      <c r="P153" s="2158"/>
+      <c r="Q153" s="2159" t="s">
+        <v>46</v>
+      </c>
+      <c r="R153" s="2160" t="s">
+        <v>89</v>
+      </c>
+      <c r="S153" s="2161" t="s">
+        <v>46</v>
+      </c>
+      <c r="T153" s="2162" t="s">
+        <v>89</v>
+      </c>
+      <c r="U153" s="2163"/>
+      <c r="V153" s="2164"/>
+    </row>
+    <row r="154" spans="2:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B154" s="2144"/>
+      <c r="C154" s="2145"/>
+      <c r="D154" s="2146"/>
+      <c r="E154" s="2147"/>
+      <c r="F154" s="2148"/>
+      <c r="G154" s="2169" t="s">
+        <v>5</v>
+      </c>
+      <c r="H154" s="2170" t="s">
+        <v>195</v>
+      </c>
+      <c r="I154" s="2151"/>
+      <c r="J154" s="2152"/>
+      <c r="K154" s="2153" t="s">
+        <v>195</v>
+      </c>
+      <c r="L154" s="2154" t="s">
+        <v>28</v>
+      </c>
+      <c r="M154" s="2155"/>
+      <c r="N154" s="2156"/>
+      <c r="O154" s="2157"/>
+      <c r="P154" s="2158"/>
+      <c r="Q154" s="2171"/>
+      <c r="R154" s="2172"/>
+      <c r="S154" s="2173"/>
+      <c r="T154" s="2174"/>
+      <c r="U154" s="2163"/>
+      <c r="V154" s="2164"/>
+    </row>
+    <row r="155" spans="2:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B155" s="2144"/>
+      <c r="C155" s="2145"/>
+      <c r="D155" s="2146"/>
+      <c r="E155" s="2147"/>
+      <c r="F155" s="2148"/>
+      <c r="G155" s="2149"/>
+      <c r="H155" s="2150"/>
+      <c r="I155" s="2151"/>
+      <c r="J155" s="2152"/>
+      <c r="K155" s="2153" t="s">
+        <v>196</v>
+      </c>
+      <c r="L155" s="2154" t="s">
+        <v>195</v>
+      </c>
+      <c r="M155" s="2155"/>
+      <c r="N155" s="2156"/>
+      <c r="O155" s="2157"/>
+      <c r="P155" s="2158"/>
+      <c r="Q155" s="2159" t="s">
+        <v>196</v>
+      </c>
+      <c r="R155" s="2160" t="s">
+        <v>195</v>
+      </c>
+      <c r="S155" s="2161" t="s">
+        <v>196</v>
+      </c>
+      <c r="T155" s="2162" t="s">
+        <v>195</v>
+      </c>
+      <c r="U155" s="2163"/>
+      <c r="V155" s="2164"/>
+    </row>
+    <row r="156" spans="2:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B156" s="2175"/>
+      <c r="C156" s="2176"/>
+      <c r="D156" s="2177"/>
+      <c r="E156" s="2178"/>
+      <c r="F156" s="2179"/>
+      <c r="G156" s="2180"/>
+      <c r="H156" s="2181"/>
+      <c r="I156" s="2182" t="s">
+        <v>25</v>
+      </c>
+      <c r="J156" s="2183" t="s">
+        <v>36</v>
+      </c>
+      <c r="K156" s="2184"/>
+      <c r="L156" s="2185"/>
+      <c r="M156" s="2186"/>
+      <c r="N156" s="2187"/>
+      <c r="O156" s="2188"/>
+      <c r="P156" s="2189"/>
+      <c r="Q156" s="2190" t="s">
+        <v>25</v>
+      </c>
+      <c r="R156" s="2191" t="s">
+        <v>36</v>
+      </c>
+      <c r="S156" s="2192" t="s">
+        <v>25</v>
+      </c>
+      <c r="T156" s="2193" t="s">
+        <v>36</v>
+      </c>
+      <c r="U156" s="2194"/>
+      <c r="V156" s="2195"/>
+    </row>
+    <row r="157" spans="2:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B157" s="2196" t="s">
+        <v>18</v>
+      </c>
+      <c r="C157" s="2197">
+        <v>60</v>
+      </c>
+      <c r="D157" s="2198"/>
+      <c r="E157" s="2199">
+        <v>32.799999999999997</v>
+      </c>
+      <c r="F157" s="2200"/>
+      <c r="G157" s="2201">
+        <v>11422.73</v>
+      </c>
+      <c r="H157" s="2202"/>
+      <c r="I157" s="2203">
+        <v>218</v>
+      </c>
+      <c r="J157" s="2204"/>
+      <c r="K157" s="2205">
+        <v>0</v>
+      </c>
+      <c r="L157" s="2206"/>
+      <c r="M157" s="2207">
+        <v>48.48</v>
+      </c>
+      <c r="N157" s="2208"/>
+      <c r="O157" s="2209">
+        <v>0</v>
+      </c>
+      <c r="P157" s="2210"/>
+      <c r="Q157" s="2211">
+        <v>0</v>
+      </c>
+      <c r="R157" s="2212">
+        <v>78.94</v>
+      </c>
+      <c r="S157" s="2213">
+        <v>0</v>
+      </c>
+      <c r="T157" s="2214">
+        <v>78.94</v>
+      </c>
+      <c r="U157" s="2215">
+        <v>11782.01</v>
+      </c>
+      <c r="V157" s="2216" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="158" spans="2:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B158" s="2217" t="s">
+        <v>20</v>
+      </c>
+      <c r="C158" s="2218"/>
+      <c r="D158" s="2219"/>
+      <c r="E158" s="2220"/>
+      <c r="F158" s="2221"/>
+      <c r="G158" s="2222"/>
+      <c r="H158" s="2223"/>
+      <c r="I158" s="2224"/>
+      <c r="J158" s="2225"/>
+      <c r="K158" s="2226"/>
+      <c r="L158" s="2227"/>
+      <c r="M158" s="2228"/>
+      <c r="N158" s="2229"/>
+      <c r="O158" s="2230"/>
+      <c r="P158" s="2231"/>
+      <c r="Q158" s="2232">
+        <v>0</v>
+      </c>
+      <c r="R158" s="2233">
+        <v>2538.8200000000002</v>
+      </c>
+      <c r="S158" s="2234">
+        <v>3700</v>
+      </c>
+      <c r="T158" s="2235">
+        <v>3038.82</v>
+      </c>
+      <c r="U158" s="2236"/>
+      <c r="V158" s="2237"/>
+    </row>
+    <row r="159" spans="2:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B159" s="2248" t="s">
+        <v>21</v>
+      </c>
+      <c r="C159" s="2249">
+        <v>60</v>
+      </c>
+      <c r="D159" s="2250" t="s">
+        <v>19</v>
+      </c>
+      <c r="E159" s="2251">
+        <v>32.799999999999997</v>
+      </c>
+      <c r="F159" s="2252" t="s">
+        <v>19</v>
+      </c>
+      <c r="G159" s="2253">
+        <v>11422.73</v>
+      </c>
+      <c r="H159" s="2254" t="s">
+        <v>19</v>
+      </c>
+      <c r="I159" s="2255">
+        <v>218</v>
+      </c>
+      <c r="J159" s="2256" t="s">
+        <v>19</v>
+      </c>
+      <c r="K159" s="2257">
+        <v>0</v>
+      </c>
+      <c r="L159" s="2258" t="s">
+        <v>19</v>
+      </c>
+      <c r="M159" s="2259">
+        <v>48.48</v>
+      </c>
+      <c r="N159" s="2260" t="s">
+        <v>19</v>
+      </c>
+      <c r="O159" s="2261">
+        <v>0</v>
+      </c>
+      <c r="P159" s="2262" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q159" s="2263"/>
+      <c r="R159" s="2264"/>
+      <c r="S159" s="2265"/>
+      <c r="T159" s="2266"/>
+      <c r="U159" s="2267">
+        <v>11782.01</v>
+      </c>
+      <c r="V159" s="2268" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="160" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B160" s="2269" t="s">
+        <v>197</v>
+      </c>
+      <c r="C160" s="2270"/>
+      <c r="D160" s="2271"/>
+      <c r="E160" s="2272"/>
+      <c r="F160" s="2273"/>
+      <c r="G160" s="2274"/>
+      <c r="H160" s="2275"/>
+      <c r="I160" s="2276" t="s">
+        <v>50</v>
+      </c>
+      <c r="J160" s="2277" t="s">
+        <v>136</v>
+      </c>
+      <c r="K160" s="2278"/>
+      <c r="L160" s="2279"/>
+      <c r="M160" s="2280"/>
+      <c r="N160" s="2281"/>
+      <c r="O160" s="2282"/>
+      <c r="P160" s="2283"/>
+      <c r="Q160" s="2284" t="s">
+        <v>50</v>
+      </c>
+      <c r="R160" s="2285" t="s">
+        <v>136</v>
+      </c>
+      <c r="S160" s="2286" t="s">
+        <v>50</v>
+      </c>
+      <c r="T160" s="2287" t="s">
+        <v>136</v>
+      </c>
+      <c r="U160" s="2288"/>
+      <c r="V160" s="2289"/>
+    </row>
+    <row r="161" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B161" s="2290"/>
+      <c r="C161" s="2291"/>
+      <c r="D161" s="2292"/>
+      <c r="E161" s="2293"/>
+      <c r="F161" s="2294"/>
+      <c r="G161" s="2295" t="s">
+        <v>5</v>
+      </c>
+      <c r="H161" s="2296" t="s">
+        <v>198</v>
+      </c>
+      <c r="I161" s="2297"/>
+      <c r="J161" s="2298"/>
+      <c r="K161" s="2299" t="s">
+        <v>198</v>
+      </c>
+      <c r="L161" s="2300" t="s">
+        <v>28</v>
+      </c>
+      <c r="M161" s="2301"/>
+      <c r="N161" s="2302"/>
+      <c r="O161" s="2303"/>
+      <c r="P161" s="2304"/>
+      <c r="Q161" s="2305"/>
+      <c r="R161" s="2306"/>
+      <c r="S161" s="2307"/>
+      <c r="T161" s="2308"/>
+      <c r="U161" s="2309"/>
+      <c r="V161" s="2310"/>
+    </row>
+    <row r="162" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B162" s="2290"/>
+      <c r="C162" s="2291"/>
+      <c r="D162" s="2292"/>
+      <c r="E162" s="2293"/>
+      <c r="F162" s="2294"/>
+      <c r="G162" s="2311"/>
+      <c r="H162" s="2312"/>
+      <c r="I162" s="2297"/>
+      <c r="J162" s="2298"/>
+      <c r="K162" s="2299" t="s">
+        <v>46</v>
+      </c>
+      <c r="L162" s="2300" t="s">
+        <v>198</v>
+      </c>
+      <c r="M162" s="2301"/>
+      <c r="N162" s="2302"/>
+      <c r="O162" s="2303"/>
+      <c r="P162" s="2304"/>
+      <c r="Q162" s="2313" t="s">
+        <v>46</v>
+      </c>
+      <c r="R162" s="2314" t="s">
+        <v>198</v>
+      </c>
+      <c r="S162" s="2315" t="s">
+        <v>46</v>
+      </c>
+      <c r="T162" s="2316" t="s">
+        <v>198</v>
+      </c>
+      <c r="U162" s="2309"/>
+      <c r="V162" s="2310"/>
+    </row>
+    <row r="163" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B163" s="2290"/>
+      <c r="C163" s="2291"/>
+      <c r="D163" s="2292"/>
+      <c r="E163" s="2293"/>
+      <c r="F163" s="2294"/>
+      <c r="G163" s="2311"/>
+      <c r="H163" s="2312"/>
+      <c r="I163" s="2317" t="s">
+        <v>50</v>
+      </c>
+      <c r="J163" s="2318" t="s">
+        <v>165</v>
+      </c>
+      <c r="K163" s="2319"/>
+      <c r="L163" s="2320"/>
+      <c r="M163" s="2301"/>
+      <c r="N163" s="2302"/>
+      <c r="O163" s="2303"/>
+      <c r="P163" s="2304"/>
+      <c r="Q163" s="2313" t="s">
+        <v>50</v>
+      </c>
+      <c r="R163" s="2314" t="s">
+        <v>165</v>
+      </c>
+      <c r="S163" s="2315" t="s">
+        <v>50</v>
+      </c>
+      <c r="T163" s="2316" t="s">
+        <v>165</v>
+      </c>
+      <c r="U163" s="2309"/>
+      <c r="V163" s="2310"/>
+    </row>
+    <row r="164" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B164" s="2321"/>
+      <c r="C164" s="2322"/>
+      <c r="D164" s="2323"/>
+      <c r="E164" s="2324"/>
+      <c r="F164" s="2325"/>
+      <c r="G164" s="2326"/>
+      <c r="H164" s="2327"/>
+      <c r="I164" s="2328"/>
+      <c r="J164" s="2329"/>
+      <c r="K164" s="2330"/>
+      <c r="L164" s="2331"/>
+      <c r="M164" s="2332" t="s">
+        <v>65</v>
+      </c>
+      <c r="N164" s="2333" t="s">
+        <v>61</v>
+      </c>
+      <c r="O164" s="2334"/>
+      <c r="P164" s="2335"/>
+      <c r="Q164" s="2336" t="s">
+        <v>65</v>
+      </c>
+      <c r="R164" s="2337" t="s">
+        <v>61</v>
+      </c>
+      <c r="S164" s="2338" t="s">
+        <v>65</v>
+      </c>
+      <c r="T164" s="2339" t="s">
+        <v>61</v>
+      </c>
+      <c r="U164" s="2340"/>
+      <c r="V164" s="2341"/>
+    </row>
+    <row r="165" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B165" s="2342" t="s">
+        <v>18</v>
+      </c>
+      <c r="C165" s="2343">
+        <v>60</v>
+      </c>
+      <c r="D165" s="2344"/>
+      <c r="E165" s="2345">
+        <v>32.799999999999997</v>
+      </c>
+      <c r="F165" s="2346"/>
+      <c r="G165" s="2347">
+        <v>11339.73</v>
+      </c>
+      <c r="H165" s="2348"/>
+      <c r="I165" s="2349">
+        <v>192.2</v>
+      </c>
+      <c r="J165" s="2350"/>
+      <c r="K165" s="2351">
+        <v>0</v>
+      </c>
+      <c r="L165" s="2352"/>
+      <c r="M165" s="2353">
+        <v>0</v>
+      </c>
+      <c r="N165" s="2354"/>
+      <c r="O165" s="2355">
+        <v>0</v>
+      </c>
+      <c r="P165" s="2356"/>
+      <c r="Q165" s="2357">
+        <v>0</v>
+      </c>
+      <c r="R165" s="2358">
+        <v>157.28</v>
+      </c>
+      <c r="S165" s="2359">
+        <v>0</v>
+      </c>
+      <c r="T165" s="2360">
+        <v>157.28</v>
+      </c>
+      <c r="U165" s="2361">
+        <v>11624.73</v>
+      </c>
+      <c r="V165" s="2362" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="166" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B166" s="2363" t="s">
+        <v>20</v>
+      </c>
+      <c r="C166" s="2364"/>
+      <c r="D166" s="2365"/>
+      <c r="E166" s="2366"/>
+      <c r="F166" s="2367"/>
+      <c r="G166" s="2368"/>
+      <c r="H166" s="2369"/>
+      <c r="I166" s="2370"/>
+      <c r="J166" s="2371"/>
+      <c r="K166" s="2372"/>
+      <c r="L166" s="2373"/>
+      <c r="M166" s="2374"/>
+      <c r="N166" s="2375"/>
+      <c r="O166" s="2376"/>
+      <c r="P166" s="2377"/>
+      <c r="Q166" s="2378">
+        <v>0</v>
+      </c>
+      <c r="R166" s="2379">
+        <v>2696.1</v>
+      </c>
+      <c r="S166" s="2380">
+        <v>3700</v>
+      </c>
+      <c r="T166" s="2381">
+        <v>3196.1</v>
+      </c>
+      <c r="U166" s="2382"/>
+      <c r="V166" s="2383"/>
+    </row>
+    <row r="167" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B167" s="2384" t="s">
+        <v>21</v>
+      </c>
+      <c r="C167" s="2385">
+        <v>60</v>
+      </c>
+      <c r="D167" s="2386" t="s">
+        <v>19</v>
+      </c>
+      <c r="E167" s="2387">
+        <v>32.799999999999997</v>
+      </c>
+      <c r="F167" s="2388" t="s">
+        <v>19</v>
+      </c>
+      <c r="G167" s="2389">
+        <v>11339.73</v>
+      </c>
+      <c r="H167" s="2390" t="s">
+        <v>19</v>
+      </c>
+      <c r="I167" s="2391">
+        <v>192.2</v>
+      </c>
+      <c r="J167" s="2392" t="s">
+        <v>19</v>
+      </c>
+      <c r="K167" s="2393">
+        <v>0</v>
+      </c>
+      <c r="L167" s="2394" t="s">
+        <v>19</v>
+      </c>
+      <c r="M167" s="2395">
+        <v>0</v>
+      </c>
+      <c r="N167" s="2396" t="s">
+        <v>19</v>
+      </c>
+      <c r="O167" s="2397">
+        <v>0</v>
+      </c>
+      <c r="P167" s="2398" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q167" s="2399"/>
+      <c r="R167" s="2400"/>
+      <c r="S167" s="2401"/>
+      <c r="T167" s="2402"/>
+      <c r="U167" s="2403">
+        <v>11624.73</v>
+      </c>
+      <c r="V167" s="2404" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="168" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B168" s="2269" t="s">
+        <v>199</v>
+      </c>
+      <c r="C168" s="2270"/>
+      <c r="D168" s="2271"/>
+      <c r="E168" s="2272"/>
+      <c r="F168" s="2273"/>
+      <c r="G168" s="2405" t="s">
+        <v>5</v>
+      </c>
+      <c r="H168" s="2406" t="s">
+        <v>200</v>
+      </c>
+      <c r="I168" s="2407"/>
+      <c r="J168" s="2408"/>
+      <c r="K168" s="2409" t="s">
+        <v>200</v>
+      </c>
+      <c r="L168" s="2410" t="s">
+        <v>28</v>
+      </c>
+      <c r="M168" s="2280"/>
+      <c r="N168" s="2281"/>
+      <c r="O168" s="2282"/>
+      <c r="P168" s="2283"/>
+      <c r="Q168" s="2411"/>
+      <c r="R168" s="2412"/>
+      <c r="S168" s="2413"/>
+      <c r="T168" s="2414"/>
+      <c r="U168" s="2288"/>
+      <c r="V168" s="2289"/>
+    </row>
+    <row r="169" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B169" s="2290"/>
+      <c r="C169" s="2291"/>
+      <c r="D169" s="2292"/>
+      <c r="E169" s="2293"/>
+      <c r="F169" s="2294"/>
+      <c r="G169" s="2311"/>
+      <c r="H169" s="2312"/>
+      <c r="I169" s="2297"/>
+      <c r="J169" s="2298"/>
+      <c r="K169" s="2299" t="s">
+        <v>29</v>
+      </c>
+      <c r="L169" s="2300" t="s">
+        <v>200</v>
+      </c>
+      <c r="M169" s="2301"/>
+      <c r="N169" s="2302"/>
+      <c r="O169" s="2303"/>
+      <c r="P169" s="2304"/>
+      <c r="Q169" s="2313" t="s">
+        <v>29</v>
+      </c>
+      <c r="R169" s="2314" t="s">
+        <v>200</v>
+      </c>
+      <c r="S169" s="2315" t="s">
+        <v>29</v>
+      </c>
+      <c r="T169" s="2316" t="s">
+        <v>200</v>
+      </c>
+      <c r="U169" s="2309"/>
+      <c r="V169" s="2310"/>
+    </row>
+    <row r="170" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B170" s="2290"/>
+      <c r="C170" s="2291"/>
+      <c r="D170" s="2292"/>
+      <c r="E170" s="2293"/>
+      <c r="F170" s="2294"/>
+      <c r="G170" s="2295" t="s">
+        <v>138</v>
+      </c>
+      <c r="H170" s="2296" t="s">
+        <v>201</v>
+      </c>
+      <c r="I170" s="2297"/>
+      <c r="J170" s="2298"/>
+      <c r="K170" s="2319"/>
+      <c r="L170" s="2320"/>
+      <c r="M170" s="2301"/>
+      <c r="N170" s="2302"/>
+      <c r="O170" s="2415" t="s">
+        <v>201</v>
+      </c>
+      <c r="P170" s="2416" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q170" s="2305"/>
+      <c r="R170" s="2306"/>
+      <c r="S170" s="2307"/>
+      <c r="T170" s="2308"/>
+      <c r="U170" s="2309"/>
+      <c r="V170" s="2310"/>
+    </row>
+    <row r="171" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B171" s="2290"/>
+      <c r="C171" s="2291"/>
+      <c r="D171" s="2292"/>
+      <c r="E171" s="2293"/>
+      <c r="F171" s="2294"/>
+      <c r="G171" s="2311"/>
+      <c r="H171" s="2312"/>
+      <c r="I171" s="2297"/>
+      <c r="J171" s="2298"/>
+      <c r="K171" s="2319"/>
+      <c r="L171" s="2320"/>
+      <c r="M171" s="2301"/>
+      <c r="N171" s="2302"/>
+      <c r="O171" s="2415" t="s">
+        <v>46</v>
+      </c>
+      <c r="P171" s="2416" t="s">
+        <v>201</v>
+      </c>
+      <c r="Q171" s="2313" t="s">
+        <v>46</v>
+      </c>
+      <c r="R171" s="2314" t="s">
+        <v>201</v>
+      </c>
+      <c r="S171" s="2315" t="s">
+        <v>46</v>
+      </c>
+      <c r="T171" s="2316" t="s">
+        <v>201</v>
+      </c>
+      <c r="U171" s="2309"/>
+      <c r="V171" s="2310"/>
+    </row>
+    <row r="172" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B172" s="2290"/>
+      <c r="C172" s="2291"/>
+      <c r="D172" s="2292"/>
+      <c r="E172" s="2293"/>
+      <c r="F172" s="2294"/>
+      <c r="G172" s="2311"/>
+      <c r="H172" s="2312"/>
+      <c r="I172" s="2317" t="s">
+        <v>50</v>
+      </c>
+      <c r="J172" s="2318" t="s">
+        <v>136</v>
+      </c>
+      <c r="K172" s="2319"/>
+      <c r="L172" s="2320"/>
+      <c r="M172" s="2301"/>
+      <c r="N172" s="2302"/>
+      <c r="O172" s="2303"/>
+      <c r="P172" s="2304"/>
+      <c r="Q172" s="2313" t="s">
+        <v>50</v>
+      </c>
+      <c r="R172" s="2314" t="s">
+        <v>136</v>
+      </c>
+      <c r="S172" s="2315" t="s">
+        <v>50</v>
+      </c>
+      <c r="T172" s="2316" t="s">
+        <v>136</v>
+      </c>
+      <c r="U172" s="2309"/>
+      <c r="V172" s="2310"/>
+    </row>
+    <row r="173" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B173" s="2290"/>
+      <c r="C173" s="2291"/>
+      <c r="D173" s="2292"/>
+      <c r="E173" s="2293"/>
+      <c r="F173" s="2294"/>
+      <c r="G173" s="2295" t="s">
+        <v>138</v>
+      </c>
+      <c r="H173" s="2296" t="s">
+        <v>173</v>
+      </c>
+      <c r="I173" s="2297"/>
+      <c r="J173" s="2298"/>
+      <c r="K173" s="2319"/>
+      <c r="L173" s="2320"/>
+      <c r="M173" s="2301"/>
+      <c r="N173" s="2302"/>
+      <c r="O173" s="2415" t="s">
+        <v>173</v>
+      </c>
+      <c r="P173" s="2416" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q173" s="2305"/>
+      <c r="R173" s="2306"/>
+      <c r="S173" s="2307"/>
+      <c r="T173" s="2308"/>
+      <c r="U173" s="2309"/>
+      <c r="V173" s="2310"/>
+    </row>
+    <row r="174" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B174" s="2290"/>
+      <c r="C174" s="2291"/>
+      <c r="D174" s="2292"/>
+      <c r="E174" s="2293"/>
+      <c r="F174" s="2294"/>
+      <c r="G174" s="2311"/>
+      <c r="H174" s="2312"/>
+      <c r="I174" s="2297"/>
+      <c r="J174" s="2298"/>
+      <c r="K174" s="2319"/>
+      <c r="L174" s="2320"/>
+      <c r="M174" s="2301"/>
+      <c r="N174" s="2302"/>
+      <c r="O174" s="2415" t="s">
+        <v>46</v>
+      </c>
+      <c r="P174" s="2416" t="s">
+        <v>173</v>
+      </c>
+      <c r="Q174" s="2313" t="s">
+        <v>46</v>
+      </c>
+      <c r="R174" s="2314" t="s">
+        <v>173</v>
+      </c>
+      <c r="S174" s="2315" t="s">
+        <v>46</v>
+      </c>
+      <c r="T174" s="2316" t="s">
+        <v>173</v>
+      </c>
+      <c r="U174" s="2309"/>
+      <c r="V174" s="2310"/>
+    </row>
+    <row r="175" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B175" s="2290"/>
+      <c r="C175" s="2291"/>
+      <c r="D175" s="2292"/>
+      <c r="E175" s="2293"/>
+      <c r="F175" s="2294"/>
+      <c r="G175" s="2311"/>
+      <c r="H175" s="2312"/>
+      <c r="I175" s="2317" t="s">
+        <v>50</v>
+      </c>
+      <c r="J175" s="2318" t="s">
+        <v>165</v>
+      </c>
+      <c r="K175" s="2319"/>
+      <c r="L175" s="2320"/>
+      <c r="M175" s="2301"/>
+      <c r="N175" s="2302"/>
+      <c r="O175" s="2303"/>
+      <c r="P175" s="2304"/>
+      <c r="Q175" s="2313" t="s">
+        <v>50</v>
+      </c>
+      <c r="R175" s="2314" t="s">
+        <v>165</v>
+      </c>
+      <c r="S175" s="2315" t="s">
+        <v>50</v>
+      </c>
+      <c r="T175" s="2316" t="s">
+        <v>165</v>
+      </c>
+      <c r="U175" s="2309"/>
+      <c r="V175" s="2310"/>
+    </row>
+    <row r="176" spans="2:22" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B176" s="2290"/>
+      <c r="C176" s="2291"/>
+      <c r="D176" s="2292"/>
+      <c r="E176" s="2293"/>
+      <c r="F176" s="2294"/>
+      <c r="G176" s="2295" t="s">
+        <v>5</v>
+      </c>
+      <c r="H176" s="2296" t="s">
+        <v>202</v>
+      </c>
+      <c r="I176" s="2297"/>
+      <c r="J176" s="2298"/>
+      <c r="K176" s="2299" t="s">
+        <v>202</v>
+      </c>
+      <c r="L176" s="2300" t="s">
+        <v>28</v>
+      </c>
+      <c r="M176" s="2301"/>
+      <c r="N176" s="2302"/>
+      <c r="O176" s="2303"/>
+      <c r="P176" s="2304"/>
+      <c r="Q176" s="2305"/>
+      <c r="R176" s="2306"/>
+      <c r="S176" s="2307"/>
+      <c r="T176" s="2308"/>
+      <c r="U176" s="2309"/>
+      <c r="V176" s="2310"/>
+    </row>
+    <row r="177" spans="2:23" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B177" s="2321"/>
+      <c r="C177" s="2322"/>
+      <c r="D177" s="2323"/>
+      <c r="E177" s="2324"/>
+      <c r="F177" s="2325"/>
+      <c r="G177" s="2326"/>
+      <c r="H177" s="2327"/>
+      <c r="I177" s="2328"/>
+      <c r="J177" s="2329"/>
+      <c r="K177" s="2417" t="s">
+        <v>33</v>
+      </c>
+      <c r="L177" s="2418" t="s">
+        <v>202</v>
+      </c>
+      <c r="M177" s="2419"/>
+      <c r="N177" s="2420"/>
+      <c r="O177" s="2334"/>
+      <c r="P177" s="2335"/>
+      <c r="Q177" s="2336" t="s">
+        <v>33</v>
+      </c>
+      <c r="R177" s="2337" t="s">
+        <v>202</v>
+      </c>
+      <c r="S177" s="2338" t="s">
+        <v>33</v>
+      </c>
+      <c r="T177" s="2339" t="s">
+        <v>202</v>
+      </c>
+      <c r="U177" s="2340"/>
+      <c r="V177" s="2341"/>
+      <c r="W177" s="1098" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="178" spans="2:23" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B178" s="2342" t="s">
+        <v>18</v>
+      </c>
+      <c r="C178" s="2343">
+        <v>60</v>
+      </c>
+      <c r="D178" s="2344"/>
+      <c r="E178" s="2345">
+        <v>32.799999999999997</v>
+      </c>
+      <c r="F178" s="2346"/>
+      <c r="G178" s="2347">
+        <v>11113.6</v>
+      </c>
+      <c r="H178" s="2348"/>
+      <c r="I178" s="2349">
+        <v>166.4</v>
+      </c>
+      <c r="J178" s="2350"/>
+      <c r="K178" s="2351">
+        <v>0</v>
+      </c>
+      <c r="L178" s="2352"/>
+      <c r="M178" s="2353">
+        <v>0</v>
+      </c>
+      <c r="N178" s="2354"/>
+      <c r="O178" s="2355">
+        <v>0</v>
+      </c>
+      <c r="P178" s="2356"/>
+      <c r="Q178" s="2357">
+        <v>0</v>
+      </c>
+      <c r="R178" s="2358">
+        <v>251.93</v>
+      </c>
+      <c r="S178" s="2359">
+        <v>0</v>
+      </c>
+      <c r="T178" s="2360">
+        <v>251.93</v>
+      </c>
+      <c r="U178" s="2361">
+        <v>11372.8</v>
+      </c>
+      <c r="V178" s="2362" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="179" spans="2:23" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B179" s="2363" t="s">
+        <v>20</v>
+      </c>
+      <c r="C179" s="2364"/>
+      <c r="D179" s="2365"/>
+      <c r="E179" s="2366"/>
+      <c r="F179" s="2367"/>
+      <c r="G179" s="2368"/>
+      <c r="H179" s="2369"/>
+      <c r="I179" s="2370"/>
+      <c r="J179" s="2371"/>
+      <c r="K179" s="2372"/>
+      <c r="L179" s="2373"/>
+      <c r="M179" s="2374"/>
+      <c r="N179" s="2375"/>
+      <c r="O179" s="2376"/>
+      <c r="P179" s="2377"/>
+      <c r="Q179" s="2378">
+        <v>0</v>
+      </c>
+      <c r="R179" s="2379">
+        <v>2948.03</v>
+      </c>
+      <c r="S179" s="2380">
+        <v>3700</v>
+      </c>
+      <c r="T179" s="2381">
+        <v>3448.03</v>
+      </c>
+      <c r="U179" s="2382"/>
+      <c r="V179" s="2383"/>
+    </row>
+    <row r="180" spans="2:23" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B180" s="2384" t="s">
+        <v>21</v>
+      </c>
+      <c r="C180" s="2385">
+        <v>60</v>
+      </c>
+      <c r="D180" s="2386" t="s">
+        <v>19</v>
+      </c>
+      <c r="E180" s="2387">
+        <v>32.799999999999997</v>
+      </c>
+      <c r="F180" s="2388" t="s">
+        <v>19</v>
+      </c>
+      <c r="G180" s="2389">
+        <v>11113.6</v>
+      </c>
+      <c r="H180" s="2390" t="s">
+        <v>19</v>
+      </c>
+      <c r="I180" s="2391">
+        <v>166.4</v>
+      </c>
+      <c r="J180" s="2392" t="s">
+        <v>19</v>
+      </c>
+      <c r="K180" s="2393">
+        <v>0</v>
+      </c>
+      <c r="L180" s="2394" t="s">
+        <v>19</v>
+      </c>
+      <c r="M180" s="2395">
+        <v>0</v>
+      </c>
+      <c r="N180" s="2396" t="s">
+        <v>19</v>
+      </c>
+      <c r="O180" s="2397">
+        <v>0</v>
+      </c>
+      <c r="P180" s="2398" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q180" s="2399"/>
+      <c r="R180" s="2400"/>
+      <c r="S180" s="2401"/>
+      <c r="T180" s="2402"/>
+      <c r="U180" s="2403">
+        <v>11372.8</v>
+      </c>
+      <c r="V180" s="2404" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>